<commit_message>
Fix report generation and image paths
</commit_message>
<xml_diff>
--- a/scripts/output/analysis_results.xlsx
+++ b/scripts/output/analysis_results.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Horner" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Derivative" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LogLog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horner" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Derivative" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LogLog" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -50,7 +47,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -58,19 +55,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
Add Savitzky-Golay smoothing to Bourdet derivative and reduce synthetic data noise
</commit_message>
<xml_diff>
--- a/scripts/output/analysis_results.xlsx
+++ b/scripts/output/analysis_results.xlsx
@@ -1015,12 +1015,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1039,6 +1040,11 @@
           <t>Bourdet Derivative</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Bourdet Derivative (Smoothed)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1048,6 +1054,7 @@
         <v>3002.483570765056</v>
       </c>
       <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1057,7 +1064,10 @@
         <v>2985.211218741119</v>
       </c>
       <c r="C3" t="n">
-        <v>-97.32266685391598</v>
+        <v>-81.50461533423048</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-81.50461533423048</v>
       </c>
     </row>
     <row r="4">
@@ -1068,7 +1078,10 @@
         <v>2975.043523184454</v>
       </c>
       <c r="C4" t="n">
-        <v>-70.53912217726409</v>
+        <v>-103.6664869302823</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-103.6664869302823</v>
       </c>
     </row>
     <row r="5">
@@ -1079,7 +1092,10 @@
         <v>2965.322770022966</v>
       </c>
       <c r="C5" t="n">
-        <v>-115.6383122965612</v>
+        <v>-111.164527155619</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-111.164527155619</v>
       </c>
     </row>
     <row r="6">
@@ -1090,7 +1106,10 @@
         <v>2942.439394114284</v>
       </c>
       <c r="C6" t="n">
-        <v>-131.1610539086692</v>
+        <v>-113.5192248900983</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-113.5192248900983</v>
       </c>
     </row>
     <row r="7">
@@ -1101,7 +1120,10 @@
         <v>2928.34201645013</v>
       </c>
       <c r="C7" t="n">
-        <v>-67.84232368810873</v>
+        <v>-84.5201741585777</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-84.5201741585777</v>
       </c>
     </row>
     <row r="8">
@@ -1112,7 +1134,10 @@
         <v>2923.311305559389</v>
       </c>
       <c r="C8" t="n">
-        <v>-82.23843685939413</v>
+        <v>-89.7909717784224</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-89.7909717784224</v>
       </c>
     </row>
     <row r="9">
@@ -1123,7 +1148,10 @@
         <v>2905.154955374591</v>
       </c>
       <c r="C9" t="n">
-        <v>-136.3307864915676</v>
+        <v>-115.6895475246959</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-115.6895475246959</v>
       </c>
     </row>
     <row r="10">
@@ -1134,7 +1162,10 @@
         <v>2884.872950046127</v>
       </c>
       <c r="C10" t="n">
-        <v>-103.9878582650078</v>
+        <v>-114.3461922103868</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-114.3461922103868</v>
       </c>
     </row>
     <row r="11">
@@ -1145,7 +1176,10 @@
         <v>2875.835662440707</v>
       </c>
       <c r="C11" t="n">
-        <v>-99.8925924735962</v>
+        <v>-105.4037538298405</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-105.4037538298405</v>
       </c>
     </row>
     <row r="12">
@@ -1156,7 +1190,10 @@
         <v>2856.70831400569</v>
       </c>
       <c r="C12" t="n">
-        <v>-117.8807000484581</v>
+        <v>-101.817151658379</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-101.817151658379</v>
       </c>
     </row>
     <row r="13">
@@ -1167,7 +1204,10 @@
         <v>2842.599293948876</v>
       </c>
       <c r="C13" t="n">
-        <v>-87.49100943120193</v>
+        <v>-105.8755032237716</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-105.8755032237716</v>
       </c>
     </row>
     <row r="14">
@@ -1178,7 +1218,10 @@
         <v>2832.040294321533</v>
       </c>
       <c r="C14" t="n">
-        <v>-125.6704136143582</v>
+        <v>-120.6594812591433</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-120.6594812591433</v>
       </c>
     </row>
     <row r="15">
@@ -1189,7 +1232,10 @@
         <v>2807.166621987389</v>
       </c>
       <c r="C15" t="n">
-        <v>-134.8800446771445</v>
+        <v>-119.6834119599489</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-119.6834119599489</v>
       </c>
     </row>
     <row r="16">
@@ -1200,7 +1246,10 @@
         <v>2794.010974295088</v>
       </c>
       <c r="C16" t="n">
-        <v>-76.04191217628531</v>
+        <v>-95.12455105103231</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-95.12455105103231</v>
       </c>
     </row>
     <row r="17">
@@ -1211,7 +1260,10 @@
         <v>2785.726666058424</v>
       </c>
       <c r="C17" t="n">
-        <v>-87.37207403578658</v>
+        <v>-77.49238667811201</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-77.49238667811201</v>
       </c>
     </row>
     <row r="18">
@@ -1222,7 +1274,10 @@
         <v>2769.376488349932</v>
       </c>
       <c r="C18" t="n">
-        <v>-84.45580130760511</v>
+        <v>-86.91228615287206</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-86.91228615287206</v>
       </c>
     </row>
     <row r="19">
@@ -1233,7 +1288,10 @@
         <v>2761.914420861556</v>
       </c>
       <c r="C19" t="n">
-        <v>-98.14138421656727</v>
+        <v>-108.9558956430238</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-108.9558956430238</v>
       </c>
     </row>
     <row r="20">
@@ -1244,7 +1302,10 @@
         <v>2741.705604067948</v>
       </c>
       <c r="C20" t="n">
-        <v>-130.6181231260513</v>
+        <v>-102.9381158000882</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-102.9381158000882</v>
       </c>
     </row>
     <row r="21">
@@ -1255,7 +1316,10 @@
         <v>2725.086746185853</v>
       </c>
       <c r="C21" t="n">
-        <v>-57.90601842410861</v>
+        <v>-80.87188554422913</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-80.87188554422913</v>
       </c>
     </row>
     <row r="22">
@@ -1266,7 +1330,10 @@
         <v>2725.379048784112</v>
       </c>
       <c r="C22" t="n">
-        <v>-78.95848930169346</v>
+        <v>-79.40147543897008</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-79.40147543897008</v>
       </c>
     </row>
     <row r="23">
@@ -1277,7 +1344,10 @@
         <v>2702.824463684048</v>
       </c>
       <c r="C23" t="n">
-        <v>-124.7938385483538</v>
+        <v>-114.7963177499478</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-114.7963177499478</v>
       </c>
     </row>
     <row r="24">
@@ -1288,7 +1358,10 @@
         <v>2690.193526456895</v>
       </c>
       <c r="C24" t="n">
-        <v>-121.2621973520766</v>
+        <v>-126.6864159682264</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-126.6864159682264</v>
       </c>
     </row>
     <row r="25">
@@ -1299,7 +1372,10 @@
         <v>2668.634684749363</v>
       </c>
       <c r="C25" t="n">
-        <v>-110.8514395489184</v>
+        <v>-100.1762753558693</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-100.1762753558693</v>
       </c>
     </row>
     <row r="26">
@@ -1310,7 +1386,10 @@
         <v>2658.93905230478</v>
       </c>
       <c r="C26" t="n">
-        <v>-72.76688845318733</v>
+        <v>-92.76124339980461</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-92.76124339980461</v>
       </c>
     </row>
     <row r="27">
@@ -1321,7 +1400,10 @@
         <v>2648.11811912293</v>
       </c>
       <c r="C27" t="n">
-        <v>-110.7574496314307</v>
+        <v>-94.18454596903757</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-94.18454596903757</v>
       </c>
     </row>
     <row r="28">
@@ -1332,7 +1414,10 @@
         <v>2627.711078534245</v>
       </c>
       <c r="C28" t="n">
-        <v>-95.30455427299388</v>
+        <v>-99.38120884383785</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-99.38120884383785</v>
       </c>
     </row>
     <row r="29">
@@ -1343,7 +1428,10 @@
         <v>2621.24707676006</v>
       </c>
       <c r="C29" t="n">
-        <v>-90.24017629514184</v>
+        <v>-96.7837805785329</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-96.7837805785329</v>
       </c>
     </row>
     <row r="30">
@@ -1354,7 +1442,10 @@
         <v>2602.267933465712</v>
       </c>
       <c r="C30" t="n">
-        <v>-111.8353196219594</v>
+        <v>-106.070221552956</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-106.070221552956</v>
       </c>
     </row>
     <row r="31">
@@ -1365,7 +1456,10 @@
         <v>2589.715198413315</v>
       </c>
       <c r="C31" t="n">
-        <v>-100.0189382046353</v>
+        <v>-92.76206253773083</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-92.76206253773083</v>
       </c>
     </row>
     <row r="32">
@@ -1376,7 +1470,10 @@
         <v>2574.06767434811</v>
       </c>
       <c r="C32" t="n">
-        <v>-61.97946346606388</v>
+        <v>-72.52526135908641</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-72.52526135908641</v>
       </c>
     </row>
     <row r="33">
@@ -1387,7 +1484,10 @@
         <v>2572.240138578777</v>
       </c>
       <c r="C33" t="n">
-        <v>-89.56887627635807</v>
+        <v>-100.8601190953792</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-100.8601190953792</v>
       </c>
     </row>
     <row r="34">
@@ -1398,7 +1498,10 @@
         <v>2548.813801779518</v>
       </c>
       <c r="C34" t="n">
-        <v>-151.604848753701</v>
+        <v>-119.4165245512974</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-119.4165245512974</v>
       </c>
     </row>
     <row r="35">
@@ -1409,7 +1512,10 @@
         <v>2529.495273505403</v>
       </c>
       <c r="C35" t="n">
-        <v>-85.17388679436189</v>
+        <v>-111.4449848687881</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-111.4449848687881</v>
       </c>
     </row>
     <row r="36">
@@ -1420,7 +1526,10 @@
         <v>2524.799092957674</v>
       </c>
       <c r="C36" t="n">
-        <v>-102.8929453226509</v>
+        <v>-94.50685213014553</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-94.50685213014553</v>
       </c>
     </row>
     <row r="37">
@@ -1431,7 +1540,10 @@
         <v>2500.484690394278</v>
       </c>
       <c r="C37" t="n">
-        <v>-110.8828350612384</v>
+        <v>-109.7044181536041</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-109.7044181536041</v>
       </c>
     </row>
     <row r="38">
@@ -1442,7 +1554,10 @@
         <v>2493.535766866132</v>
       </c>
       <c r="C38" t="n">
-        <v>-113.1021206453567</v>
+        <v>-122.4706225101267</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-122.4706225101267</v>
       </c>
     </row>
     <row r="39">
@@ -1453,7 +1568,10 @@
         <v>2468.595638518685</v>
       </c>
       <c r="C39" t="n">
-        <v>-127.2575639659711</v>
+        <v>-106.8281294683832</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-106.8281294683832</v>
       </c>
     </row>
     <row r="40">
@@ -1464,7 +1582,10 @@
         <v>2457.655599140567</v>
       </c>
       <c r="C40" t="n">
-        <v>-61.75673849173003</v>
+        <v>-77.04286141152753</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-77.04286141152753</v>
       </c>
     </row>
     <row r="41">
@@ -1475,7 +1596,10 @@
         <v>2451.18337581138</v>
       </c>
       <c r="C41" t="n">
-        <v>-63.35062016314013</v>
+        <v>-65.60725414361686</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-65.60725414361686</v>
       </c>
     </row>
     <row r="42">
@@ -1486,7 +1610,10 @@
         <v>2439.793942778986</v>
       </c>
       <c r="C42" t="n">
-        <v>-100.452084189737</v>
+        <v>-95.40702723424931</v>
+      </c>
+      <c r="D42" t="n">
+        <v>-95.40702723424931</v>
       </c>
     </row>
     <row r="43">
@@ -1497,7 +1624,10 @@
         <v>2422.860991531934</v>
       </c>
       <c r="C43" t="n">
-        <v>-115.1466093421605</v>
+        <v>-111.4543780008282</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-111.4543780008282</v>
       </c>
     </row>
     <row r="44">
@@ -1508,7 +1638,10 @@
         <v>2407.328448961019</v>
       </c>
       <c r="C44" t="n">
-        <v>-108.3786722050725</v>
+        <v>-116.873954918418</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-116.873954918418</v>
       </c>
     </row>
     <row r="45">
@@ -1519,7 +1652,10 @@
         <v>2392.303712141989</v>
       </c>
       <c r="C45" t="n">
-        <v>-124.1687816786776</v>
+        <v>-117.4067367878427</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-117.4067367878427</v>
       </c>
     </row>
     <row r="46">
@@ -1530,7 +1666,10 @@
         <v>2372.319160915073</v>
       </c>
       <c r="C46" t="n">
-        <v>-107.4258150074819</v>
+        <v>-107.6872805556338</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-107.6872805556338</v>
       </c>
     </row>
     <row r="47">
@@ -1541,7 +1680,10 @@
         <v>2362.015090071912</v>
       </c>
       <c r="C47" t="n">
-        <v>-81.94917316239848</v>
+        <v>-82.12516076754801</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-82.12516076754801</v>
       </c>
     </row>
     <row r="48">
@@ -1552,7 +1694,10 @@
         <v>2349.213657506062</v>
       </c>
       <c r="C48" t="n">
-        <v>-68.48782571923478</v>
+        <v>-68.69201842371272</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-68.69201842371272</v>
       </c>
     </row>
     <row r="49">
@@ -1563,7 +1708,10 @@
         <v>2342.70500273893</v>
       </c>
       <c r="C49" t="n">
-        <v>-85.73755352705308</v>
+        <v>-92.60328775324399</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-92.60328775324399</v>
       </c>
     </row>
     <row r="50">
@@ -1574,7 +1722,10 @@
         <v>2325.040023302653</v>
       </c>
       <c r="C50" t="n">
-        <v>-150.0118892160059</v>
+        <v>-146.5449899854975</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-146.5449899854975</v>
       </c>
     </row>
     <row r="51">
@@ -1585,6 +1736,7 @@
         <v>2300.409271324973</v>
       </c>
       <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>